<commit_message>
Add CAMBIOS_Y_PRUEBAS guide, update docs for final component list, ignore trained model
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/02_Plan_Gestion_Riesgos.xlsx
+++ b/docs/02_Plan_Gestion_Riesgos.xlsx
@@ -157,7 +157,7 @@
     <t>Lecturas inestables del sensor de frecuencia cardiaca MAX30102 por movimiento</t>
   </si>
   <si>
-    <t>Leonardo Nágera</t>
+    <t>Leonardo Nájera</t>
   </si>
   <si>
     <t>m</t>
@@ -169,7 +169,7 @@
     <t>A: Abierto, el riesgo está latente.</t>
   </si>
   <si>
-    <t>Daño del ESP32 por mezcla de voltajes (3.3V lógica / 12V actuadores)</t>
+    <t>Daño del ESP32 por mezcla de voltajes (3.3V lógica / 12V y 5V actuadores)</t>
   </si>
   <si>
     <t>b</t>
@@ -538,10 +538,10 @@
     <t>Fecha:</t>
   </si>
   <si>
-    <t>Daño del ESP32 por mezcla de voltajes (3.3V / 12V)</t>
-  </si>
-  <si>
-    <t>El ventilador y el relé operan a 12V mientras el ESP32 trabaja a 3.3V; una conexión incorrecta (sin optoacoplador o sin tierra común) puede dañar permanentemente el microcontrolador prestado por el laboratorio.</t>
+    <t>Daño del ESP32 por mezcla de voltajes (3.3V / 12V / 5V)</t>
+  </si>
+  <si>
+    <t>El ventilador (12V, regulado por el módulo D4184) y el módulo vibratorio (5V) operan a voltajes distintos al del ESP32 (3.3V); una conexión incorrecta (sin tierra común entre las fuentes y el ESP32, o sin los diodos 1N5819 de protección) puede dañar permanentemente el microcontrolador prestado por el laboratorio.</t>
   </si>
   <si>
     <t>13-oct-26</t>
@@ -571,7 +571,7 @@
     <t>Pendiente</t>
   </si>
   <si>
-    <t>Unir las tierras (GND) de la fuente de 12V y el ESP32 antes de probar</t>
+    <t>Unir las tierras (GND) de las fuentes de 12V y 5V y el ESP32 antes de probar</t>
   </si>
   <si>
     <t>Aunque el sprint de construcción es de solo 14 días, un retraso acumulado en tareas de la ruta crítica o imprevistos no resueltos durante las 6 semanas de margen podrían impedir tener el prototipo listo para la demostración final.</t>

</xml_diff>